<commit_message>
Simplify upgrade descriptions in workbook
Co-authored-by: TWBSY <nnmnsalmon@gmail.com>
</commit_message>
<xml_diff>
--- a/gacha_design_upgrades_items_ko.xlsx
+++ b/gacha_design_upgrades_items_ko.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>전역 판매가 보너스</t>
+          <t>모든 아이템을 조금 더 비싸게 팔 수 있어요.</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>후반용 전역 보너스</t>
+          <t>후반에는 전체 판매가를 더 크게 올려줘요.</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>N 전용</t>
+          <t>N등급은 기본값도 올라가고, 싸게 팔리는 날에도 덜 손해 봐요.</t>
         </is>
       </c>
     </row>
@@ -678,17 +678,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>R 기본 판매가 +10%/레벨; R 시세계수 최소값 +0.03</t>
+          <t>R 기본 판매가 +10%/레벨; 최저 가격선 +3%p</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>R 기본 판매가 +40%; 시세계수 최소값 +0.12</t>
+          <t>R 기본 판매가 +40%; 최저 가격선 +12%p</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>R 전용</t>
+          <t>R등급은 좋은 날엔 더 비싸고, 나쁜 날에도 덜 싸게 팔려요.</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>SR 기본 판매가 +8%/레벨; SR 시세계수 최소값 +0.02</t>
+          <t>SR 기본 판매가 +8%/레벨; 최저 가격선 +2%p</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SR 기본 판매가 +32%; 시세계수 최소값 +0.08</t>
+          <t>SR 기본 판매가 +32%; 최저 가격선 +8%p</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>SR 전용</t>
+          <t>SR등급은 비싼 날이 더 많고, 싸게 팔리는 날이 줄어요.</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>확률 재분배</t>
+          <t>낮은 등급이 줄고, 높은 등급이 조금 더 잘 나와요.</t>
         </is>
       </c>
     </row>
@@ -831,17 +831,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>모든 등급 시세계수 최소값 +0.05/레벨</t>
+          <t>모든 등급 최저 가격선 +5%p/레벨</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>시세계수 최소값 +0.20</t>
+          <t>최저 가격선 +20%p</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>폭락 방지</t>
+          <t>오늘 가격이 너무 싸게 떨어지는 걸 막아줘요.</t>
         </is>
       </c>
     </row>
@@ -886,17 +886,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>시세계수 ≥1.5 판매 시 추가 +5%/레벨</t>
+          <t>오늘 가격이 1.5배 이상일 때 추가 +5%/레벨</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>최대 +25%</t>
+          <t>추가 +25%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>호황 타이밍 강화</t>
+          <t>오늘 가격이 아주 비싼 날엔 추가 보너스가 붙어요.</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>기본: 3초 내 연속 판매 시 콤보+1, 기본 최대 콤보 5, 콤보×2% 보너스(기본 최대 +10%)</t>
+          <t>빠르게 연속으로 팔수록 보너스가 커져요.</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>기본: 최근 50개 판매 중 31~50개면 +5%</t>
+          <t>최근에 많이 팔수록 더 큰 보너스를 받아요.</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>일회성 업그레이드</t>
+          <t>가끔 나타나는 특별한 상인을 열어줘요.</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1225,7 +1224,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1277,7 +1275,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1329,7 +1326,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1381,7 +1377,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1433,7 +1428,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1485,7 +1479,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1537,7 +1530,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1589,7 +1581,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1697,7 +1688,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1749,7 +1739,6 @@
           <t>예</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>